<commit_message>
Add single-formula selection to contract price workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFaw3CrmucU3qXrStYrfnC
</commit_message>
<xml_diff>
--- a/Выбор_по_договору.xlsx
+++ b/Выбор_по_договору.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="16">
   <si>
     <t xml:space="preserve">ID аналогов</t>
   </si>
@@ -62,6 +62,12 @@
   </si>
   <si>
     <t xml:space="preserve">RAM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Одной формулой: материал</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Одной формулой: всё вместе</t>
   </si>
 </sst>
 </file>
@@ -145,16 +151,24 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -423,264 +437,278 @@
   <dimension ref="M1:W9"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="11.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="9.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="19.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="12.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="23.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="36.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="35.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="11.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="9.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="19.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="12.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="23.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="36.22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="35.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="26"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M1" s="0" t="s">
+    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="N1" s="0" t="s">
+      <c r="N1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="O1" s="0" t="s">
+      <c r="O1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="P1" s="0" t="s">
+      <c r="P1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="Q1" s="0" t="s">
+      <c r="Q1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="R1" s="0" t="s">
+      <c r="R1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="S1" s="0" t="s">
+      <c r="S1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="W1" s="2" t="n">
+      <c r="W1" s="3" t="n">
         <f aca="false" t="array" ref="W1:W1">MIN(IF(((P2:P9="RAM")+(P2:P9="KON"))&gt;0,Q2:Q9))</f>
         <v>765.36</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="M2" s="0" t="n">
+    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="M2" s="1" t="n">
         <v>99008177</v>
       </c>
-      <c r="N2" s="0" t="n">
+      <c r="N2" s="1" t="n">
         <v>147185</v>
       </c>
-      <c r="O2" s="0" t="s">
+      <c r="O2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="P2" s="0" t="s">
+      <c r="P2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="Q2" s="0" t="n">
+      <c r="Q2" s="1" t="n">
         <v>3772.23</v>
       </c>
-      <c r="R2" s="0" t="n">
+      <c r="R2" s="1" t="n">
         <v>242</v>
       </c>
-      <c r="S2" s="0" t="n">
+      <c r="S2" s="1" t="n">
         <v>158</v>
       </c>
-      <c r="T2" s="0" t="str">
+      <c r="T2" s="1" t="str">
         <f aca="false">IF(AND(OR(P2="RAM",P2="KON"),Q2=$W$1),"Выбрать","")</f>
         <v/>
       </c>
-      <c r="V2" s="1" t="s">
+      <c r="V2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="W2" s="0" t="n">
+      <c r="W2" s="1" t="n">
         <f aca="false" t="array" ref="W2:W2">INDEX(N2:N9,MATCH(1,(Q2:Q9=W1)*((P2:P9="RAM")+(P2:P9="KON")),0))</f>
         <v>298733</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N3" s="0" t="n">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="N3" s="1" t="n">
         <v>298654</v>
       </c>
-      <c r="O3" s="0" t="s">
+      <c r="O3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="P3" s="0" t="s">
+      <c r="P3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="Q3" s="0" t="n">
+      <c r="Q3" s="1" t="n">
         <v>594.94</v>
       </c>
-      <c r="R3" s="0" t="n">
+      <c r="R3" s="1" t="n">
         <v>212</v>
       </c>
-      <c r="S3" s="0" t="n">
+      <c r="S3" s="1" t="n">
         <v>128</v>
       </c>
-      <c r="T3" s="0" t="str">
+      <c r="T3" s="1" t="str">
         <f aca="false">IF(AND(OR(P3="RAM",P3="KON"),Q3=$W$1),"Выбрать","")</f>
         <v/>
       </c>
-      <c r="V3" s="1" t="s">
+      <c r="V3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="W3" s="0" t="str">
+      <c r="W3" s="1" t="str">
         <f aca="false" t="array" ref="W3:W3">INDEX(O2:O9,MATCH(1,(Q2:Q9=W1)*((P2:P9="RAM")+(P2:P9="KON")),0))</f>
         <v>РВД</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N4" s="0" t="n">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="N4" s="1" t="n">
         <v>298733</v>
       </c>
-      <c r="O4" s="0" t="s">
+      <c r="O4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="P4" s="0" t="s">
+      <c r="P4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="Q4" s="0" t="n">
+      <c r="Q4" s="1" t="n">
         <v>765.36</v>
       </c>
-      <c r="R4" s="0" t="n">
+      <c r="R4" s="1" t="n">
         <v>143</v>
       </c>
-      <c r="S4" s="0" t="n">
+      <c r="S4" s="1" t="n">
         <v>59</v>
       </c>
-      <c r="T4" s="0" t="str">
+      <c r="T4" s="1" t="str">
         <f aca="false">IF(AND(OR(P4="RAM",P4="KON"),Q4=$W$1),"Выбрать","")</f>
         <v>Выбрать</v>
       </c>
-      <c r="V4" s="1" t="s">
+      <c r="V4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="W4" s="0" t="str">
+      <c r="W4" s="1" t="str">
         <f aca="false" t="array" ref="W4:W4">INDEX(P2:P9,MATCH(1,(Q2:Q9=W1)*((P2:P9="RAM")+(P2:P9="KON")),0))</f>
         <v>RAM</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N5" s="0" t="n">
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="N5" s="1" t="n">
         <v>508788</v>
       </c>
-      <c r="O5" s="0" t="s">
+      <c r="O5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="P5" s="0" t="s">
+      <c r="P5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="Q5" s="0" t="n">
+      <c r="Q5" s="1" t="n">
         <v>368.56</v>
       </c>
-      <c r="R5" s="0" t="n">
+      <c r="R5" s="1" t="n">
         <v>202</v>
       </c>
-      <c r="S5" s="0" t="n">
+      <c r="S5" s="1" t="n">
         <v>118</v>
       </c>
-      <c r="T5" s="0" t="str">
+      <c r="T5" s="1" t="str">
         <f aca="false">IF(AND(OR(P5="RAM",P5="KON"),Q5=$W$1),"Выбрать","")</f>
         <v/>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N6" s="0" t="n">
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="N6" s="1" t="n">
         <v>509811</v>
       </c>
-      <c r="O6" s="0" t="s">
+      <c r="O6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="P6" s="0" t="s">
+      <c r="P6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="Q6" s="0" t="n">
+      <c r="Q6" s="1" t="n">
         <v>873.5</v>
       </c>
-      <c r="R6" s="0" t="n">
+      <c r="R6" s="1" t="n">
         <v>165</v>
       </c>
-      <c r="S6" s="0" t="n">
+      <c r="S6" s="1" t="n">
         <v>81</v>
       </c>
-      <c r="T6" s="0" t="str">
+      <c r="T6" s="1" t="str">
         <f aca="false">IF(AND(OR(P6="RAM",P6="KON"),Q6=$W$1),"Выбрать","")</f>
         <v/>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N7" s="0" t="n">
+      <c r="V6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="W6" s="1" t="n">
+        <f aca="false" t="array" ref="W6:W6">INDEX(N2:N9,MATCH(MIN(IF(((P2:P9="RAM")+(P2:P9="KON")),Q2:Q9)),IF(((P2:P9="RAM")+(P2:P9="KON")),Q2:Q9),0))</f>
+        <v>298733</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="N7" s="1" t="n">
         <v>519150</v>
       </c>
-      <c r="O7" s="0" t="s">
+      <c r="O7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="P7" s="0" t="s">
+      <c r="P7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="Q7" s="0" t="n">
+      <c r="Q7" s="1" t="n">
         <v>1229.03</v>
       </c>
-      <c r="R7" s="0" t="n">
+      <c r="R7" s="1" t="n">
         <v>202</v>
       </c>
-      <c r="S7" s="0" t="n">
+      <c r="S7" s="1" t="n">
         <v>118</v>
       </c>
-      <c r="T7" s="0" t="str">
+      <c r="T7" s="1" t="str">
         <f aca="false">IF(AND(OR(P7="RAM",P7="KON"),Q7=$W$1),"Выбрать","")</f>
         <v/>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N8" s="0" t="n">
+      <c r="V7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="W7" s="1" t="str">
+        <f aca="false" t="array" ref="W7:W7">INDEX(N2:N9,MATCH(MIN(IF(((P2:P9="RAM")+(P2:P9="KON")),Q2:Q9)),IF(((P2:P9="RAM")+(P2:P9="KON")),Q2:Q9),0))&amp;" | "&amp;INDEX(P2:P9,MATCH(MIN(IF(((P2:P9="RAM")+(P2:P9="KON")),Q2:Q9)),IF(((P2:P9="RAM")+(P2:P9="KON")),Q2:Q9),0))&amp;" | "&amp;TEXT(MIN(IF(((P2:P9="RAM")+(P2:P9="KON")),Q2:Q9)),"# ##0.00")</f>
+        <v>298733 | RAM |  765.36</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="N8" s="1" t="n">
         <v>526401</v>
       </c>
-      <c r="O8" s="0" t="s">
+      <c r="O8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="P8" s="0" t="s">
+      <c r="P8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="Q8" s="0" t="n">
+      <c r="Q8" s="1" t="n">
         <v>752.39</v>
       </c>
-      <c r="R8" s="0" t="n">
+      <c r="R8" s="1" t="n">
         <v>212</v>
       </c>
-      <c r="S8" s="0" t="n">
+      <c r="S8" s="1" t="n">
         <v>128</v>
       </c>
-      <c r="T8" s="0" t="str">
+      <c r="T8" s="1" t="str">
         <f aca="false">IF(AND(OR(P8="RAM",P8="KON"),Q8=$W$1),"Выбрать","")</f>
         <v/>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N9" s="0" t="n">
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="N9" s="1" t="n">
         <v>1520422</v>
       </c>
-      <c r="O9" s="0" t="s">
+      <c r="O9" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="P9" s="0" t="s">
+      <c r="P9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="Q9" s="0" t="n">
+      <c r="Q9" s="1" t="n">
         <v>2735.52</v>
       </c>
-      <c r="R9" s="0" t="e">
+      <c r="R9" s="1" t="e">
         <f aca="false">#N/A</f>
         <v>#N/A</v>
       </c>
-      <c r="S9" s="0" t="e">
+      <c r="S9" s="1" t="e">
         <f aca="false">#N/A</f>
         <v>#N/A</v>
       </c>
-      <c r="T9" s="0" t="str">
+      <c r="T9" s="1" t="str">
         <f aca="false">IF(AND(OR(P9="RAM",P9="KON"),Q9=$W$1),"Выбрать","")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Make column T selection formula self-contained
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFaw3CrmucU3qXrStYrfnC
</commit_message>
<xml_diff>
--- a/Выбор_по_договору.xlsx
+++ b/Выбор_по_договору.xlsx
@@ -151,7 +151,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -165,10 +165,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -504,7 +500,7 @@
         <v>158</v>
       </c>
       <c r="T2" s="1" t="str">
-        <f aca="false">IF(AND(OR(P2="RAM",P2="KON"),Q2=$W$1),"Выбрать","")</f>
+        <f aca="false" t="array" ref="T2:T2">IF(AND(OR(P2="RAM",P2="KON"),Q2=MIN(IF(($P$2:$P$9="RAM")+($P$2:$P$9="KON"),$Q$2:$Q$9))),"Выбрать","")</f>
         <v/>
       </c>
       <c r="V2" s="2" t="s">
@@ -535,7 +531,7 @@
         <v>128</v>
       </c>
       <c r="T3" s="1" t="str">
-        <f aca="false">IF(AND(OR(P3="RAM",P3="KON"),Q3=$W$1),"Выбрать","")</f>
+        <f aca="false" t="array" ref="T3:T3">IF(AND(OR(P3="RAM",P3="KON"),Q3=MIN(IF(($P$2:$P$9="RAM")+($P$2:$P$9="KON"),$Q$2:$Q$9))),"Выбрать","")</f>
         <v/>
       </c>
       <c r="V3" s="2" t="s">
@@ -566,7 +562,7 @@
         <v>59</v>
       </c>
       <c r="T4" s="1" t="str">
-        <f aca="false">IF(AND(OR(P4="RAM",P4="KON"),Q4=$W$1),"Выбрать","")</f>
+        <f aca="false" t="array" ref="T4:T4">IF(AND(OR(P4="RAM",P4="KON"),Q4=MIN(IF(($P$2:$P$9="RAM")+($P$2:$P$9="KON"),$Q$2:$Q$9))),"Выбрать","")</f>
         <v>Выбрать</v>
       </c>
       <c r="V4" s="2" t="s">
@@ -597,7 +593,7 @@
         <v>118</v>
       </c>
       <c r="T5" s="1" t="str">
-        <f aca="false">IF(AND(OR(P5="RAM",P5="KON"),Q5=$W$1),"Выбрать","")</f>
+        <f aca="false" t="array" ref="T5:T5">IF(AND(OR(P5="RAM",P5="KON"),Q5=MIN(IF(($P$2:$P$9="RAM")+($P$2:$P$9="KON"),$Q$2:$Q$9))),"Выбрать","")</f>
         <v/>
       </c>
     </row>
@@ -621,10 +617,10 @@
         <v>81</v>
       </c>
       <c r="T6" s="1" t="str">
-        <f aca="false">IF(AND(OR(P6="RAM",P6="KON"),Q6=$W$1),"Выбрать","")</f>
+        <f aca="false" t="array" ref="T6:T6">IF(AND(OR(P6="RAM",P6="KON"),Q6=MIN(IF(($P$2:$P$9="RAM")+($P$2:$P$9="KON"),$Q$2:$Q$9))),"Выбрать","")</f>
         <v/>
       </c>
-      <c r="V6" s="4" t="s">
+      <c r="V6" s="2" t="s">
         <v>14</v>
       </c>
       <c r="W6" s="1" t="n">
@@ -652,10 +648,10 @@
         <v>118</v>
       </c>
       <c r="T7" s="1" t="str">
-        <f aca="false">IF(AND(OR(P7="RAM",P7="KON"),Q7=$W$1),"Выбрать","")</f>
+        <f aca="false" t="array" ref="T7:T7">IF(AND(OR(P7="RAM",P7="KON"),Q7=MIN(IF(($P$2:$P$9="RAM")+($P$2:$P$9="KON"),$Q$2:$Q$9))),"Выбрать","")</f>
         <v/>
       </c>
-      <c r="V7" s="4" t="s">
+      <c r="V7" s="2" t="s">
         <v>15</v>
       </c>
       <c r="W7" s="1" t="str">
@@ -683,7 +679,7 @@
         <v>128</v>
       </c>
       <c r="T8" s="1" t="str">
-        <f aca="false">IF(AND(OR(P8="RAM",P8="KON"),Q8=$W$1),"Выбрать","")</f>
+        <f aca="false" t="array" ref="T8:T8">IF(AND(OR(P8="RAM",P8="KON"),Q8=MIN(IF(($P$2:$P$9="RAM")+($P$2:$P$9="KON"),$Q$2:$Q$9))),"Выбрать","")</f>
         <v/>
       </c>
     </row>
@@ -709,7 +705,7 @@
         <v>#N/A</v>
       </c>
       <c r="T9" s="1" t="str">
-        <f aca="false">IF(AND(OR(P9="RAM",P9="KON"),Q9=$W$1),"Выбрать","")</f>
+        <f aca="false" t="array" ref="T9:T9">IF(AND(OR(P9="RAM",P9="KON"),Q9=MIN(IF(($P$2:$P$9="RAM")+($P$2:$P$9="KON"),$Q$2:$Q$9))),"Выбрать","")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Use non-array COUNTIFS formula in column T
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JFaw3CrmucU3qXrStYrfnC
</commit_message>
<xml_diff>
--- a/Выбор_по_договору.xlsx
+++ b/Выбор_по_договору.xlsx
@@ -500,7 +500,7 @@
         <v>158</v>
       </c>
       <c r="T2" s="1" t="str">
-        <f aca="false" t="array" ref="T2:T2">IF(AND(OR(P2="RAM",P2="KON"),Q2=MIN(IF(($P$2:$P$9="RAM")+($P$2:$P$9="KON"),$Q$2:$Q$9))),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P2="RAM",P2="KON"),COUNTIFS($P$2:$P$9,"RAM",$Q$2:$Q$9,"&lt;"&amp;Q2)+COUNTIFS($P$2:$P$9,"KON",$Q$2:$Q$9,"&lt;"&amp;Q2)=0),"Выбрать","")</f>
         <v/>
       </c>
       <c r="V2" s="2" t="s">
@@ -531,7 +531,7 @@
         <v>128</v>
       </c>
       <c r="T3" s="1" t="str">
-        <f aca="false" t="array" ref="T3:T3">IF(AND(OR(P3="RAM",P3="KON"),Q3=MIN(IF(($P$2:$P$9="RAM")+($P$2:$P$9="KON"),$Q$2:$Q$9))),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P3="RAM",P3="KON"),COUNTIFS($P$2:$P$9,"RAM",$Q$2:$Q$9,"&lt;"&amp;Q3)+COUNTIFS($P$2:$P$9,"KON",$Q$2:$Q$9,"&lt;"&amp;Q3)=0),"Выбрать","")</f>
         <v/>
       </c>
       <c r="V3" s="2" t="s">
@@ -562,7 +562,7 @@
         <v>59</v>
       </c>
       <c r="T4" s="1" t="str">
-        <f aca="false" t="array" ref="T4:T4">IF(AND(OR(P4="RAM",P4="KON"),Q4=MIN(IF(($P$2:$P$9="RAM")+($P$2:$P$9="KON"),$Q$2:$Q$9))),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P4="RAM",P4="KON"),COUNTIFS($P$2:$P$9,"RAM",$Q$2:$Q$9,"&lt;"&amp;Q4)+COUNTIFS($P$2:$P$9,"KON",$Q$2:$Q$9,"&lt;"&amp;Q4)=0),"Выбрать","")</f>
         <v>Выбрать</v>
       </c>
       <c r="V4" s="2" t="s">
@@ -593,7 +593,7 @@
         <v>118</v>
       </c>
       <c r="T5" s="1" t="str">
-        <f aca="false" t="array" ref="T5:T5">IF(AND(OR(P5="RAM",P5="KON"),Q5=MIN(IF(($P$2:$P$9="RAM")+($P$2:$P$9="KON"),$Q$2:$Q$9))),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P5="RAM",P5="KON"),COUNTIFS($P$2:$P$9,"RAM",$Q$2:$Q$9,"&lt;"&amp;Q5)+COUNTIFS($P$2:$P$9,"KON",$Q$2:$Q$9,"&lt;"&amp;Q5)=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>
@@ -617,7 +617,7 @@
         <v>81</v>
       </c>
       <c r="T6" s="1" t="str">
-        <f aca="false" t="array" ref="T6:T6">IF(AND(OR(P6="RAM",P6="KON"),Q6=MIN(IF(($P$2:$P$9="RAM")+($P$2:$P$9="KON"),$Q$2:$Q$9))),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P6="RAM",P6="KON"),COUNTIFS($P$2:$P$9,"RAM",$Q$2:$Q$9,"&lt;"&amp;Q6)+COUNTIFS($P$2:$P$9,"KON",$Q$2:$Q$9,"&lt;"&amp;Q6)=0),"Выбрать","")</f>
         <v/>
       </c>
       <c r="V6" s="2" t="s">
@@ -648,7 +648,7 @@
         <v>118</v>
       </c>
       <c r="T7" s="1" t="str">
-        <f aca="false" t="array" ref="T7:T7">IF(AND(OR(P7="RAM",P7="KON"),Q7=MIN(IF(($P$2:$P$9="RAM")+($P$2:$P$9="KON"),$Q$2:$Q$9))),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P7="RAM",P7="KON"),COUNTIFS($P$2:$P$9,"RAM",$Q$2:$Q$9,"&lt;"&amp;Q7)+COUNTIFS($P$2:$P$9,"KON",$Q$2:$Q$9,"&lt;"&amp;Q7)=0),"Выбрать","")</f>
         <v/>
       </c>
       <c r="V7" s="2" t="s">
@@ -679,7 +679,7 @@
         <v>128</v>
       </c>
       <c r="T8" s="1" t="str">
-        <f aca="false" t="array" ref="T8:T8">IF(AND(OR(P8="RAM",P8="KON"),Q8=MIN(IF(($P$2:$P$9="RAM")+($P$2:$P$9="KON"),$Q$2:$Q$9))),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P8="RAM",P8="KON"),COUNTIFS($P$2:$P$9,"RAM",$Q$2:$Q$9,"&lt;"&amp;Q8)+COUNTIFS($P$2:$P$9,"KON",$Q$2:$Q$9,"&lt;"&amp;Q8)=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>
@@ -705,7 +705,7 @@
         <v>#N/A</v>
       </c>
       <c r="T9" s="1" t="str">
-        <f aca="false" t="array" ref="T9:T9">IF(AND(OR(P9="RAM",P9="KON"),Q9=MIN(IF(($P$2:$P$9="RAM")+($P$2:$P$9="KON"),$Q$2:$Q$9))),"Выбрать","")</f>
+        <f aca="false">IF(AND(OR(P9="RAM",P9="KON"),COUNTIFS($P$2:$P$9,"RAM",$Q$2:$Q$9,"&lt;"&amp;Q9)+COUNTIFS($P$2:$P$9,"KON",$Q$2:$Q$9,"&lt;"&amp;Q9)=0),"Выбрать","")</f>
         <v/>
       </c>
     </row>

</xml_diff>